<commit_message>
distance travel bug entfernt, immobile bug entfernt
</commit_message>
<xml_diff>
--- a/code_test/ma_home/Metriken.xlsx
+++ b/code_test/ma_home/Metriken.xlsx
@@ -500,13 +500,13 @@
         <v>0.02788888888888889</v>
       </c>
       <c r="F2" t="n">
-        <v>0.3629474784426444</v>
+        <v>0.6238132566849578</v>
       </c>
       <c r="G2" t="n">
         <v>0.3972650465987284</v>
       </c>
       <c r="H2" t="n">
-        <v>0.780029669037878</v>
+        <v>3.017752702914369</v>
       </c>
       <c r="I2" t="n">
         <v>0.01479820627802691</v>

</xml_diff>

<commit_message>
acceleration count und mehr videos hinzugefügt
</commit_message>
<xml_diff>
--- a/code_test/ma_home/Metriken.xlsx
+++ b/code_test/ma_home/Metriken.xlsx
@@ -500,13 +500,13 @@
         <v>0.02788888888888889</v>
       </c>
       <c r="F2" t="n">
-        <v>0.6238132566849578</v>
+        <v>0.6157129169932932</v>
       </c>
       <c r="G2" t="n">
         <v>0.3972650465987284</v>
       </c>
       <c r="H2" t="n">
-        <v>3.017752702914369</v>
+        <v>3.310784872734607</v>
       </c>
       <c r="I2" t="n">
         <v>0.01479820627802691</v>

</xml_diff>

<commit_message>
bissl schabernack mit videos gemacht
</commit_message>
<xml_diff>
--- a/code_test/ma_home/Metriken.xlsx
+++ b/code_test/ma_home/Metriken.xlsx
@@ -500,13 +500,13 @@
         <v>0.02788888888888889</v>
       </c>
       <c r="F2" t="n">
-        <v>0.6157129169932932</v>
+        <v>0.6238132566849578</v>
       </c>
       <c r="G2" t="n">
         <v>0.3972650465987284</v>
       </c>
       <c r="H2" t="n">
-        <v>3.310784872734607</v>
+        <v>3.017752702914369</v>
       </c>
       <c r="I2" t="n">
         <v>0.01479820627802691</v>

</xml_diff>